<commit_message>
Fixing supplementary data paths
</commit_message>
<xml_diff>
--- a/scripts/other/cryptic/Activity_vs_cryptic.xlsx
+++ b/scripts/other/cryptic/Activity_vs_cryptic.xlsx
@@ -176,28 +176,148 @@
     <t>50</t>
   </si>
   <si>
+    <t>434_33</t>
+  </si>
+  <si>
+    <t>248_38</t>
+  </si>
+  <si>
+    <t>1723_59</t>
+  </si>
+  <si>
+    <t>1724_71</t>
+  </si>
+  <si>
+    <t>617_77</t>
+  </si>
+  <si>
+    <t>914_74</t>
+  </si>
+  <si>
+    <t>1091_44</t>
+  </si>
+  <si>
+    <t>1343_36</t>
+  </si>
+  <si>
+    <t>321_71</t>
+  </si>
+  <si>
+    <t>914_77</t>
+  </si>
+  <si>
+    <t>319_37</t>
+  </si>
+  <si>
+    <t>321_74</t>
+  </si>
+  <si>
+    <t>1663_69</t>
+  </si>
+  <si>
+    <t>409_46</t>
+  </si>
+  <si>
+    <t>1538_54</t>
+  </si>
+  <si>
+    <t>1815_56</t>
+  </si>
+  <si>
+    <t>1664_74</t>
+  </si>
+  <si>
+    <t>666_83</t>
+  </si>
+  <si>
+    <t>1668_52</t>
+  </si>
+  <si>
+    <t>1057_41</t>
+  </si>
+  <si>
+    <t>1723_62</t>
+  </si>
+  <si>
+    <t>245_48</t>
+  </si>
+  <si>
+    <t>279_60</t>
+  </si>
+  <si>
+    <t>1668_49</t>
+  </si>
+  <si>
+    <t>1863_75</t>
+  </si>
+  <si>
+    <t>1190_71</t>
+  </si>
+  <si>
+    <t>1248_60</t>
+  </si>
+  <si>
+    <t>1251_37</t>
+  </si>
+  <si>
+    <t>1406_54</t>
+  </si>
+  <si>
+    <t>1409_62</t>
+  </si>
+  <si>
+    <t>876_57</t>
+  </si>
+  <si>
+    <t>1344_72</t>
+  </si>
+  <si>
+    <t>706_38</t>
+  </si>
+  <si>
+    <t>848_71</t>
+  </si>
+  <si>
+    <t>1096_14</t>
+  </si>
+  <si>
+    <t>1855_60</t>
+  </si>
+  <si>
     <t>1630_70</t>
   </si>
   <si>
+    <t>851_60</t>
+  </si>
+  <si>
     <t>1631_52</t>
   </si>
   <si>
-    <t>666_83</t>
-  </si>
-  <si>
-    <t>1663_69</t>
-  </si>
-  <si>
-    <t>1664_74</t>
-  </si>
-  <si>
-    <t>319_37</t>
-  </si>
-  <si>
-    <t>321_71</t>
-  </si>
-  <si>
-    <t>321_74</t>
+    <t>738_68</t>
+  </si>
+  <si>
+    <t>1849_60</t>
+  </si>
+  <si>
+    <t>1850_66</t>
+  </si>
+  <si>
+    <t>1248_57</t>
+  </si>
+  <si>
+    <t>1409_59</t>
+  </si>
+  <si>
+    <t>1441_47</t>
+  </si>
+  <si>
+    <t>873_60</t>
+  </si>
+  <si>
+    <t>1921_77</t>
+  </si>
+  <si>
+    <t>1231_45</t>
   </si>
   <si>
     <t>453_72</t>
@@ -206,133 +326,13 @@
     <t>454_56</t>
   </si>
   <si>
-    <t>1538_54</t>
-  </si>
-  <si>
-    <t>738_68</t>
-  </si>
-  <si>
-    <t>409_46</t>
-  </si>
-  <si>
-    <t>1231_45</t>
-  </si>
-  <si>
-    <t>1668_49</t>
-  </si>
-  <si>
-    <t>1668_52</t>
-  </si>
-  <si>
-    <t>706_38</t>
-  </si>
-  <si>
-    <t>1057_41</t>
-  </si>
-  <si>
-    <t>1855_60</t>
-  </si>
-  <si>
-    <t>279_60</t>
-  </si>
-  <si>
-    <t>1190_71</t>
-  </si>
-  <si>
-    <t>1248_57</t>
-  </si>
-  <si>
-    <t>1248_60</t>
-  </si>
-  <si>
-    <t>1251_37</t>
-  </si>
-  <si>
-    <t>1406_54</t>
-  </si>
-  <si>
-    <t>1409_59</t>
-  </si>
-  <si>
-    <t>1409_62</t>
-  </si>
-  <si>
-    <t>1441_47</t>
-  </si>
-  <si>
-    <t>873_60</t>
-  </si>
-  <si>
-    <t>876_57</t>
-  </si>
-  <si>
-    <t>1849_60</t>
-  </si>
-  <si>
-    <t>1850_66</t>
-  </si>
-  <si>
-    <t>617_77</t>
-  </si>
-  <si>
-    <t>1815_56</t>
-  </si>
-  <si>
-    <t>434_33</t>
-  </si>
-  <si>
-    <t>245_48</t>
-  </si>
-  <si>
-    <t>248_38</t>
-  </si>
-  <si>
-    <t>1723_59</t>
-  </si>
-  <si>
-    <t>1723_62</t>
-  </si>
-  <si>
-    <t>1724_71</t>
-  </si>
-  <si>
-    <t>914_74</t>
-  </si>
-  <si>
-    <t>914_77</t>
-  </si>
-  <si>
-    <t>848_71</t>
-  </si>
-  <si>
-    <t>851_60</t>
-  </si>
-  <si>
-    <t>1091_44</t>
-  </si>
-  <si>
-    <t>1096_14</t>
-  </si>
-  <si>
-    <t>1343_36</t>
-  </si>
-  <si>
-    <t>1344_72</t>
-  </si>
-  <si>
-    <t>1863_75</t>
-  </si>
-  <si>
-    <t>1921_77</t>
+    <t>expressed &amp; active</t>
   </si>
   <si>
     <t>not expressed 
  or not active</t>
   </si>
   <si>
-    <t>expressed &amp; active</t>
-  </si>
-  <si>
     <t>num.ST</t>
   </si>
   <si>
@@ -345,25 +345,127 @@
     <t>num.prophages.in.cluster</t>
   </si>
   <si>
+    <t>KPN_B20_PHAGE088_M</t>
+  </si>
+  <si>
+    <t>KVV_B2_PHAGE021_M</t>
+  </si>
+  <si>
+    <t>KVV_B2_PHAGE157_M</t>
+  </si>
+  <si>
+    <t>KVV_B2_PHAGE154_M</t>
+  </si>
+  <si>
+    <t>KPN_B2_PHAGE139_M</t>
+  </si>
+  <si>
+    <t>KPN_B18_PHAGE117_M</t>
+  </si>
+  <si>
+    <t>KPN_B2_PHAGE370_L</t>
+  </si>
+  <si>
+    <t>KPN_B2_PHAGE047_M</t>
+  </si>
+  <si>
+    <t>KPN_B12_PHAGE103_M</t>
+  </si>
+  <si>
+    <t>KPN_B12_PHAGE105_M</t>
+  </si>
+  <si>
+    <t>KPN_B8_PHAGE117_M</t>
+  </si>
+  <si>
+    <t>KPN_B18_PHAGE008_M</t>
+  </si>
+  <si>
+    <t>KPN_B8_PHAGE148_M</t>
+  </si>
+  <si>
+    <t>KPN_B17_PHAGE532_M</t>
+  </si>
+  <si>
+    <t>KPN_B8_PHAGE116_M</t>
+  </si>
+  <si>
+    <t>KPN_B20_PHAGE077_M</t>
+  </si>
+  <si>
+    <t>KPN_B3_PHAGE386_M</t>
+  </si>
+  <si>
+    <t>KPN_B9_PHAGE130_M</t>
+  </si>
+  <si>
+    <t>KVV_B2_PHAGE022_M</t>
+  </si>
+  <si>
+    <t>KPN_B20_PHAGE101_M</t>
+  </si>
+  <si>
+    <t>KQS_B1_PHAGE085_M</t>
+  </si>
+  <si>
+    <t>KPN_B3_PHAGE143_M</t>
+  </si>
+  <si>
+    <t>KPN_B19_PHAGE044_M</t>
+  </si>
+  <si>
+    <t>KPN_B19_PHAGE043_M</t>
+  </si>
+  <si>
+    <t>KVV_B2_PHAGE063_M</t>
+  </si>
+  <si>
+    <t>KVV_B2_PHAGE067_M</t>
+  </si>
+  <si>
+    <t>KPN_B20_PHAGE149_M</t>
+  </si>
+  <si>
+    <t>KPN_B2_PHAGE046_M</t>
+  </si>
+  <si>
+    <t>KPN_B9_PHAGE157_M</t>
+  </si>
+  <si>
+    <t>KPN_B7_PHAGE163_M</t>
+  </si>
+  <si>
+    <t>KPN_B2_PHAGE033_M</t>
+  </si>
+  <si>
     <t>KVV_B2_PHAGE059_M</t>
   </si>
   <si>
+    <t>KPN_B7_PHAGE455_M</t>
+  </si>
+  <si>
     <t>KVV_B2_PHAGE060_M</t>
   </si>
   <si>
-    <t>KPN_B20_PHAGE077_M</t>
-  </si>
-  <si>
-    <t>KPN_B8_PHAGE117_M</t>
-  </si>
-  <si>
-    <t>KPN_B8_PHAGE116_M</t>
-  </si>
-  <si>
-    <t>KPN_B12_PHAGE105_M</t>
-  </si>
-  <si>
-    <t>KPN_B12_PHAGE103_M</t>
+    <t>KVV_B3_PHAGE120_M</t>
+  </si>
+  <si>
+    <t>KPN_B10_PHAGE393_M</t>
+  </si>
+  <si>
+    <t>KPN_B10_PHAGE394_M</t>
+  </si>
+  <si>
+    <t>KPN_B7_PHAGE137_M</t>
+  </si>
+  <si>
+    <t>KPN_B20_PHAGE148_M</t>
+  </si>
+  <si>
+    <t>KVV_B1_PHAGE047_L</t>
+  </si>
+  <si>
+    <t>KVV_B1_PHAGE111_M</t>
   </si>
   <si>
     <t>KVV_B1_PHAGE385_M</t>
@@ -372,232 +474,130 @@
     <t>KVV_B1_PHAGE181_L</t>
   </si>
   <si>
-    <t>KPN_B8_PHAGE148_M</t>
-  </si>
-  <si>
-    <t>KVV_B3_PHAGE120_M</t>
-  </si>
-  <si>
-    <t>KPN_B18_PHAGE008_M</t>
-  </si>
-  <si>
-    <t>KVV_B1_PHAGE111_M</t>
-  </si>
-  <si>
-    <t>KPN_B3_PHAGE386_M</t>
-  </si>
-  <si>
-    <t>KPN_B9_PHAGE157_M</t>
-  </si>
-  <si>
-    <t>KPN_B9_PHAGE130_M</t>
-  </si>
-  <si>
-    <t>KPN_B20_PHAGE101_M</t>
-  </si>
-  <si>
-    <t>KPN_B3_PHAGE143_M</t>
-  </si>
-  <si>
-    <t>KPN_B19_PHAGE044_M</t>
-  </si>
-  <si>
-    <t>KPN_B19_PHAGE043_M</t>
-  </si>
-  <si>
-    <t>KVV_B2_PHAGE063_M</t>
-  </si>
-  <si>
-    <t>KVV_B2_PHAGE067_M</t>
-  </si>
-  <si>
-    <t>KPN_B7_PHAGE137_M</t>
-  </si>
-  <si>
-    <t>KPN_B20_PHAGE148_M</t>
-  </si>
-  <si>
-    <t>KPN_B20_PHAGE149_M</t>
-  </si>
-  <si>
-    <t>KPN_B10_PHAGE393_M</t>
-  </si>
-  <si>
-    <t>KPN_B10_PHAGE394_M</t>
-  </si>
-  <si>
-    <t>KPN_B2_PHAGE139_M</t>
-  </si>
-  <si>
-    <t>KPN_B17_PHAGE532_M</t>
-  </si>
-  <si>
-    <t>KPN_B20_PHAGE088_M</t>
-  </si>
-  <si>
-    <t>KVV_B2_PHAGE022_M</t>
-  </si>
-  <si>
-    <t>KVV_B2_PHAGE021_M</t>
-  </si>
-  <si>
-    <t>KVV_B2_PHAGE157_M</t>
-  </si>
-  <si>
-    <t>KVV_B2_PHAGE154_M</t>
-  </si>
-  <si>
-    <t>KPN_B18_PHAGE117_M</t>
-  </si>
-  <si>
-    <t>KPN_B7_PHAGE163_M</t>
-  </si>
-  <si>
-    <t>KPN_B7_PHAGE455_M</t>
-  </si>
-  <si>
-    <t>KPN_B2_PHAGE370_L</t>
-  </si>
-  <si>
-    <t>KPN_B2_PHAGE033_M</t>
-  </si>
-  <si>
-    <t>KPN_B2_PHAGE047_M</t>
-  </si>
-  <si>
-    <t>KPN_B2_PHAGE046_M</t>
-  </si>
-  <si>
-    <t>KQS_B1_PHAGE085_M</t>
-  </si>
-  <si>
-    <t>KVV_B1_PHAGE047_L</t>
+    <t>PV3111</t>
+  </si>
+  <si>
+    <t>PV2680</t>
+  </si>
+  <si>
+    <t>PV0541</t>
+  </si>
+  <si>
+    <t>PV2642</t>
+  </si>
+  <si>
+    <t>PV3173</t>
+  </si>
+  <si>
+    <t>PV0531</t>
+  </si>
+  <si>
+    <t>PV0518</t>
+  </si>
+  <si>
+    <t>PV1002</t>
+  </si>
+  <si>
+    <t>PV1382</t>
+  </si>
+  <si>
+    <t>PV1408</t>
+  </si>
+  <si>
+    <t>PV3255</t>
+  </si>
+  <si>
+    <t>PV1041</t>
+  </si>
+  <si>
+    <t>PV0123</t>
+  </si>
+  <si>
+    <t>PV1157</t>
+  </si>
+  <si>
+    <t>PV3256</t>
+  </si>
+  <si>
+    <t>PV3118</t>
+  </si>
+  <si>
+    <t>PV0579</t>
+  </si>
+  <si>
+    <t>PV0089</t>
+  </si>
+  <si>
+    <t>PV2679</t>
+  </si>
+  <si>
+    <t>PV0010</t>
+  </si>
+  <si>
+    <t>PV0048</t>
+  </si>
+  <si>
+    <t>PV0468</t>
+  </si>
+  <si>
+    <t>PV0072</t>
+  </si>
+  <si>
+    <t>PV0136</t>
+  </si>
+  <si>
+    <t>PV0319</t>
+  </si>
+  <si>
+    <t>PV0542</t>
+  </si>
+  <si>
+    <t>PV3042</t>
+  </si>
+  <si>
+    <t>PV0086</t>
+  </si>
+  <si>
+    <t>PV0109</t>
+  </si>
+  <si>
+    <t>PV0213</t>
+  </si>
+  <si>
+    <t>PV0436</t>
   </si>
   <si>
     <t>PV2659</t>
   </si>
   <si>
+    <t>PV3337</t>
+  </si>
+  <si>
     <t>PV0428</t>
   </si>
   <si>
-    <t>PV3118</t>
-  </si>
-  <si>
-    <t>PV3255</t>
-  </si>
-  <si>
-    <t>PV3256</t>
-  </si>
-  <si>
-    <t>PV1408</t>
-  </si>
-  <si>
-    <t>PV1382</t>
+    <t>PV2492</t>
+  </si>
+  <si>
+    <t>PV0090</t>
+  </si>
+  <si>
+    <t>PV0895</t>
+  </si>
+  <si>
+    <t>PV0928</t>
+  </si>
+  <si>
+    <t>PV2067</t>
+  </si>
+  <si>
+    <t>PV1980</t>
   </si>
   <si>
     <t>PV0548</t>
   </si>
   <si>
     <t>PV2152</t>
-  </si>
-  <si>
-    <t>PV0123</t>
-  </si>
-  <si>
-    <t>PV2492</t>
-  </si>
-  <si>
-    <t>PV1041</t>
-  </si>
-  <si>
-    <t>PV1980</t>
-  </si>
-  <si>
-    <t>PV0579</t>
-  </si>
-  <si>
-    <t>PV0109</t>
-  </si>
-  <si>
-    <t>PV0089</t>
-  </si>
-  <si>
-    <t>PV0010</t>
-  </si>
-  <si>
-    <t>PV0468</t>
-  </si>
-  <si>
-    <t>PV0072</t>
-  </si>
-  <si>
-    <t>PV0136</t>
-  </si>
-  <si>
-    <t>PV0319</t>
-  </si>
-  <si>
-    <t>PV0542</t>
-  </si>
-  <si>
-    <t>PV0928</t>
-  </si>
-  <si>
-    <t>PV3042</t>
-  </si>
-  <si>
-    <t>PV0090</t>
-  </si>
-  <si>
-    <t>PV0895</t>
-  </si>
-  <si>
-    <t>PV3173</t>
-  </si>
-  <si>
-    <t>PV1157</t>
-  </si>
-  <si>
-    <t>PV3111</t>
-  </si>
-  <si>
-    <t>PV2679</t>
-  </si>
-  <si>
-    <t>PV2680</t>
-  </si>
-  <si>
-    <t>PV0541</t>
-  </si>
-  <si>
-    <t>PV2642</t>
-  </si>
-  <si>
-    <t>PV0531</t>
-  </si>
-  <si>
-    <t>PV0213</t>
-  </si>
-  <si>
-    <t>PV3337</t>
-  </si>
-  <si>
-    <t>PV0518</t>
-  </si>
-  <si>
-    <t>PV0436</t>
-  </si>
-  <si>
-    <t>PV1002</t>
-  </si>
-  <si>
-    <t>PV0086</t>
-  </si>
-  <si>
-    <t>PV0048</t>
-  </si>
-  <si>
-    <t>PV2067</t>
   </si>
   <si>
     <t>num.transposase</t>
@@ -741,7 +741,7 @@
         <v>100.0</v>
       </c>
       <c r="D7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8">
@@ -769,7 +769,7 @@
         <v>100.0</v>
       </c>
       <c r="D9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10">
@@ -783,7 +783,7 @@
         <v>100.0</v>
       </c>
       <c r="D10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="11">
@@ -839,7 +839,7 @@
         <v>100.0</v>
       </c>
       <c r="D14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="15">
@@ -853,7 +853,7 @@
         <v>100.0</v>
       </c>
       <c r="D15" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16">
@@ -867,7 +867,7 @@
         <v>100.0</v>
       </c>
       <c r="D16" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="17">
@@ -881,7 +881,7 @@
         <v>100.0</v>
       </c>
       <c r="D17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="18">
@@ -895,7 +895,7 @@
         <v>100.0</v>
       </c>
       <c r="D18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="19">
@@ -909,7 +909,7 @@
         <v>100.0</v>
       </c>
       <c r="D19" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="20">
@@ -923,7 +923,7 @@
         <v>100.0</v>
       </c>
       <c r="D20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="21">
@@ -937,7 +937,7 @@
         <v>100.0</v>
       </c>
       <c r="D21" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="22">
@@ -951,7 +951,7 @@
         <v>100.0</v>
       </c>
       <c r="D22" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="23">
@@ -979,7 +979,7 @@
         <v>100.0</v>
       </c>
       <c r="D24" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="25">
@@ -1007,7 +1007,7 @@
         <v>100.0</v>
       </c>
       <c r="D26" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="27">
@@ -1035,7 +1035,7 @@
         <v>100.0</v>
       </c>
       <c r="D28" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="29">
@@ -1049,7 +1049,7 @@
         <v>100.0</v>
       </c>
       <c r="D29" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="30">
@@ -1063,7 +1063,7 @@
         <v>100.0</v>
       </c>
       <c r="D30" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="31">
@@ -1077,7 +1077,7 @@
         <v>100.0</v>
       </c>
       <c r="D31" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="32">
@@ -1088,10 +1088,10 @@
         <v>83</v>
       </c>
       <c r="C32" t="n">
-        <v>93.43</v>
+        <v>100.0</v>
       </c>
       <c r="D32" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="33">
@@ -1102,10 +1102,10 @@
         <v>84</v>
       </c>
       <c r="C33" t="n">
-        <v>93.43</v>
+        <v>100.0</v>
       </c>
       <c r="D33" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="34">
@@ -1133,7 +1133,7 @@
         <v>100.0</v>
       </c>
       <c r="D35" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="36">
@@ -1161,7 +1161,7 @@
         <v>100.0</v>
       </c>
       <c r="D37" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="38">
@@ -1203,7 +1203,7 @@
         <v>100.0</v>
       </c>
       <c r="D40" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="41">
@@ -1217,7 +1217,7 @@
         <v>100.0</v>
       </c>
       <c r="D41" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="42">
@@ -1228,7 +1228,7 @@
         <v>93</v>
       </c>
       <c r="C42" t="n">
-        <v>100.0</v>
+        <v>93.43</v>
       </c>
       <c r="D42" t="s">
         <v>104</v>
@@ -1242,7 +1242,7 @@
         <v>94</v>
       </c>
       <c r="C43" t="n">
-        <v>100.0</v>
+        <v>93.43</v>
       </c>
       <c r="D43" t="s">
         <v>104</v>
@@ -1287,7 +1287,7 @@
         <v>100.0</v>
       </c>
       <c r="D46" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="47">
@@ -1301,7 +1301,7 @@
         <v>100.0</v>
       </c>
       <c r="D47" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="48">
@@ -1315,7 +1315,7 @@
         <v>100.0</v>
       </c>
       <c r="D48" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="49">
@@ -1329,7 +1329,7 @@
         <v>100.0</v>
       </c>
       <c r="D49" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="50">
@@ -1343,7 +1343,7 @@
         <v>100.0</v>
       </c>
       <c r="D50" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="51">
@@ -1357,7 +1357,7 @@
         <v>100.0</v>
       </c>
       <c r="D51" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -1387,10 +1387,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D2" t="n">
         <v>4.0</v>
@@ -1401,10 +1401,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>97</v>
+        <v>59</v>
       </c>
       <c r="C3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D3" t="n">
         <v>1.0</v>
@@ -1415,10 +1415,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="C4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D4" t="n">
         <v>1.0</v>
@@ -1429,10 +1429,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D5" t="n">
         <v>3.0</v>
@@ -1443,10 +1443,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="C6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D6" t="n">
         <v>1.0</v>
@@ -1457,10 +1457,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>74</v>
+        <v>95</v>
       </c>
       <c r="C7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D7" t="n">
         <v>2.0</v>
@@ -1471,10 +1471,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D8" t="n">
         <v>2.0</v>
@@ -1485,10 +1485,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D9" t="n">
         <v>3.0</v>
@@ -1499,10 +1499,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>99</v>
+        <v>60</v>
       </c>
       <c r="C10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D10" t="n">
         <v>1.0</v>
@@ -1513,10 +1513,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="C11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D11" t="n">
         <v>1.0</v>
@@ -1527,10 +1527,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C12" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D12" t="n">
         <v>3.0</v>
@@ -1541,10 +1541,10 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="C13" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D13" t="n">
         <v>3.0</v>
@@ -1555,10 +1555,10 @@
         <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D14" t="n">
         <v>3.0</v>
@@ -1569,10 +1569,10 @@
         <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="C15" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D15" t="n">
         <v>1.0</v>
@@ -1583,10 +1583,10 @@
         <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C16" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D16" t="n">
         <v>1.0</v>
@@ -1597,10 +1597,10 @@
         <v>18</v>
       </c>
       <c r="B17" t="s">
-        <v>53</v>
+        <v>89</v>
       </c>
       <c r="C17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D17" t="n">
         <v>1.0</v>
@@ -1611,10 +1611,10 @@
         <v>19</v>
       </c>
       <c r="B18" t="s">
-        <v>54</v>
+        <v>91</v>
       </c>
       <c r="C18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D18" t="n">
         <v>1.0</v>
@@ -1625,10 +1625,10 @@
         <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="C19" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D19" t="n">
         <v>1.0</v>
@@ -1639,10 +1639,10 @@
         <v>21</v>
       </c>
       <c r="B20" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="C20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D20" t="n">
         <v>1.0</v>
@@ -1653,10 +1653,10 @@
         <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="C21" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D21" t="n">
         <v>1.0</v>
@@ -1667,10 +1667,10 @@
         <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C22" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D22" t="n">
         <v>1.0</v>
@@ -1681,10 +1681,10 @@
         <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>90</v>
+        <v>55</v>
       </c>
       <c r="C23" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D23" t="n">
         <v>1.0</v>
@@ -1695,10 +1695,10 @@
         <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="C24" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D24" t="n">
         <v>1.0</v>
@@ -1709,10 +1709,10 @@
         <v>26</v>
       </c>
       <c r="B25" t="s">
-        <v>92</v>
+        <v>56</v>
       </c>
       <c r="C25" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D25" t="n">
         <v>1.0</v>
@@ -1723,10 +1723,10 @@
         <v>27</v>
       </c>
       <c r="B26" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="C26" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D26" t="n">
         <v>1.0</v>
@@ -1737,10 +1737,10 @@
         <v>28</v>
       </c>
       <c r="B27" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="C27" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D27" t="n">
         <v>7.0</v>
@@ -1751,10 +1751,10 @@
         <v>29</v>
       </c>
       <c r="B28" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="C28" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D28" t="n">
         <v>2.0</v>
@@ -1765,10 +1765,10 @@
         <v>30</v>
       </c>
       <c r="B29" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="C29" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D29" t="n">
         <v>2.0</v>
@@ -1779,10 +1779,10 @@
         <v>31</v>
       </c>
       <c r="B30" t="s">
-        <v>101</v>
+        <v>77</v>
       </c>
       <c r="C30" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D30" t="n">
         <v>2.0</v>
@@ -1793,10 +1793,10 @@
         <v>32</v>
       </c>
       <c r="B31" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C31" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D31" t="n">
         <v>1.0</v>
@@ -1807,10 +1807,10 @@
         <v>33</v>
       </c>
       <c r="B32" t="s">
-        <v>88</v>
+        <v>74</v>
       </c>
       <c r="C32" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D32" t="n">
         <v>1.0</v>
@@ -1821,10 +1821,10 @@
         <v>34</v>
       </c>
       <c r="B33" t="s">
-        <v>89</v>
+        <v>54</v>
       </c>
       <c r="C33" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D33" t="n">
         <v>1.0</v>
@@ -1835,10 +1835,10 @@
         <v>35</v>
       </c>
       <c r="B34" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C34" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D34" t="n">
         <v>2.0</v>
@@ -1849,10 +1849,10 @@
         <v>36</v>
       </c>
       <c r="B35" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C35" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D35" t="n">
         <v>1.0</v>
@@ -1863,10 +1863,10 @@
         <v>37</v>
       </c>
       <c r="B36" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C36" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D36" t="n">
         <v>1.0</v>
@@ -1877,10 +1877,10 @@
         <v>38</v>
       </c>
       <c r="B37" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C37" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D37" t="n">
         <v>1.0</v>
@@ -1891,10 +1891,10 @@
         <v>39</v>
       </c>
       <c r="B38" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C38" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D38" t="n">
         <v>1.0</v>
@@ -1905,10 +1905,10 @@
         <v>40</v>
       </c>
       <c r="B39" t="s">
-        <v>87</v>
+        <v>53</v>
       </c>
       <c r="C39" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D39" t="n">
         <v>1.0</v>
@@ -1919,10 +1919,10 @@
         <v>41</v>
       </c>
       <c r="B40" t="s">
-        <v>61</v>
+        <v>101</v>
       </c>
       <c r="C40" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D40" t="n">
         <v>3.0</v>
@@ -1933,10 +1933,10 @@
         <v>42</v>
       </c>
       <c r="B41" t="s">
-        <v>62</v>
+        <v>102</v>
       </c>
       <c r="C41" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D41" t="n">
         <v>1.0</v>
@@ -1947,10 +1947,10 @@
         <v>43</v>
       </c>
       <c r="B42" t="s">
-        <v>85</v>
+        <v>57</v>
       </c>
       <c r="C42" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D42" t="n">
         <v>1.0</v>
@@ -1961,10 +1961,10 @@
         <v>44</v>
       </c>
       <c r="B43" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="C43" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D43" t="n">
         <v>1.0</v>
@@ -1975,10 +1975,10 @@
         <v>45</v>
       </c>
       <c r="B44" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="C44" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D44" t="n">
         <v>3.0</v>
@@ -1989,10 +1989,10 @@
         <v>46</v>
       </c>
       <c r="B45" t="s">
-        <v>64</v>
+        <v>92</v>
       </c>
       <c r="C45" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D45" t="n">
         <v>1.0</v>
@@ -2003,10 +2003,10 @@
         <v>47</v>
       </c>
       <c r="B46" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="C46" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D46" t="n">
         <v>2.0</v>
@@ -2017,10 +2017,10 @@
         <v>48</v>
       </c>
       <c r="B47" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="C47" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D47" t="n">
         <v>1.0</v>
@@ -2031,10 +2031,10 @@
         <v>49</v>
       </c>
       <c r="B48" t="s">
-        <v>81</v>
+        <v>98</v>
       </c>
       <c r="C48" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D48" t="n">
         <v>2.0</v>
@@ -2045,10 +2045,10 @@
         <v>50</v>
       </c>
       <c r="B49" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C49" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D49" t="n">
         <v>1.0</v>
@@ -2059,10 +2059,10 @@
         <v>51</v>
       </c>
       <c r="B50" t="s">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="C50" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D50" t="n">
         <v>2.0</v>
@@ -2073,10 +2073,10 @@
         <v>52</v>
       </c>
       <c r="B51" t="s">
-        <v>94</v>
+        <v>62</v>
       </c>
       <c r="C51" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D51" t="n">
         <v>2.0</v>
@@ -2147,7 +2147,7 @@
         <v>153</v>
       </c>
       <c r="F3" t="n">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="4">
@@ -2167,7 +2167,7 @@
         <v>154</v>
       </c>
       <c r="F4" t="n">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="5">
@@ -2218,7 +2218,7 @@
         <v>58</v>
       </c>
       <c r="C7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D7" t="s">
         <v>114</v>
@@ -2227,7 +2227,7 @@
         <v>157</v>
       </c>
       <c r="F7" t="n">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="8">
@@ -2247,7 +2247,7 @@
         <v>158</v>
       </c>
       <c r="F8" t="n">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="9">
@@ -2258,16 +2258,16 @@
         <v>60</v>
       </c>
       <c r="C9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F9" t="n">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="10">
@@ -2278,16 +2278,16 @@
         <v>61</v>
       </c>
       <c r="C10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F10" t="n">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="11">
@@ -2301,13 +2301,13 @@
         <v>103</v>
       </c>
       <c r="D11" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="E11" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="F11" t="n">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="12">
@@ -2327,7 +2327,7 @@
         <v>161</v>
       </c>
       <c r="F12" t="n">
-        <v>8.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="13">
@@ -2341,10 +2341,10 @@
         <v>104</v>
       </c>
       <c r="D13" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E13" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="F13" t="n">
         <v>1.0</v>
@@ -2358,13 +2358,13 @@
         <v>65</v>
       </c>
       <c r="C14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D14" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F14" t="n">
         <v>1.0</v>
@@ -2378,13 +2378,13 @@
         <v>66</v>
       </c>
       <c r="C15" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E15" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F15" t="n">
         <v>1.0</v>
@@ -2398,16 +2398,16 @@
         <v>67</v>
       </c>
       <c r="C16" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D16" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E16" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F16" t="n">
-        <v>2.0</v>
+        <v>8.0</v>
       </c>
     </row>
     <row r="17">
@@ -2418,7 +2418,7 @@
         <v>68</v>
       </c>
       <c r="C17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D17" t="s">
         <v>122</v>
@@ -2427,7 +2427,7 @@
         <v>165</v>
       </c>
       <c r="F17" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="18">
@@ -2438,7 +2438,7 @@
         <v>69</v>
       </c>
       <c r="C18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D18" t="s">
         <v>123</v>
@@ -2447,7 +2447,7 @@
         <v>166</v>
       </c>
       <c r="F18" t="n">
-        <v>9.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="19">
@@ -2458,7 +2458,7 @@
         <v>70</v>
       </c>
       <c r="C19" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D19" t="s">
         <v>124</v>
@@ -2467,7 +2467,7 @@
         <v>167</v>
       </c>
       <c r="F19" t="n">
-        <v>11.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="20">
@@ -2478,7 +2478,7 @@
         <v>71</v>
       </c>
       <c r="C20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D20" t="s">
         <v>125</v>
@@ -2487,7 +2487,7 @@
         <v>168</v>
       </c>
       <c r="F20" t="n">
-        <v>43.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="21">
@@ -2498,16 +2498,16 @@
         <v>72</v>
       </c>
       <c r="C21" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E21" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F21" t="n">
-        <v>43.0</v>
+        <v>11.0</v>
       </c>
     </row>
     <row r="22">
@@ -2518,13 +2518,13 @@
         <v>73</v>
       </c>
       <c r="C22" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D22" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="E22" t="s">
-        <v>169</v>
+        <v>154</v>
       </c>
       <c r="F22" t="n">
         <v>3.0</v>
@@ -2547,7 +2547,7 @@
         <v>170</v>
       </c>
       <c r="F23" t="n">
-        <v>13.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="24">
@@ -2558,16 +2558,16 @@
         <v>75</v>
       </c>
       <c r="C24" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D24" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E24" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F24" t="n">
-        <v>13.0</v>
+        <v>43.0</v>
       </c>
     </row>
     <row r="25">
@@ -2581,13 +2581,13 @@
         <v>104</v>
       </c>
       <c r="D25" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E25" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="F25" t="n">
-        <v>8.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="26">
@@ -2598,7 +2598,7 @@
         <v>77</v>
       </c>
       <c r="C26" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D26" t="s">
         <v>129</v>
@@ -2607,7 +2607,7 @@
         <v>172</v>
       </c>
       <c r="F26" t="n">
-        <v>4.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="27">
@@ -2638,16 +2638,16 @@
         <v>79</v>
       </c>
       <c r="C28" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D28" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E28" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F28" t="n">
-        <v>3.0</v>
+        <v>13.0</v>
       </c>
     </row>
     <row r="29">
@@ -2658,16 +2658,16 @@
         <v>80</v>
       </c>
       <c r="C29" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D29" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E29" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F29" t="n">
-        <v>2.0</v>
+        <v>8.0</v>
       </c>
     </row>
     <row r="30">
@@ -2678,16 +2678,16 @@
         <v>81</v>
       </c>
       <c r="C30" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D30" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E30" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="F30" t="n">
-        <v>13.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="31">
@@ -2698,16 +2698,16 @@
         <v>82</v>
       </c>
       <c r="C31" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D31" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E31" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="F31" t="n">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="32">
@@ -2718,16 +2718,16 @@
         <v>83</v>
       </c>
       <c r="C32" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D32" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E32" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F32" t="n">
-        <v>10.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="33">
@@ -2738,16 +2738,16 @@
         <v>84</v>
       </c>
       <c r="C33" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D33" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E33" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F33" t="n">
-        <v>2.0</v>
+        <v>11.0</v>
       </c>
     </row>
     <row r="34">
@@ -2761,13 +2761,13 @@
         <v>104</v>
       </c>
       <c r="D34" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E34" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="F34" t="n">
-        <v>1.0</v>
+        <v>9.0</v>
       </c>
     </row>
     <row r="35">
@@ -2778,16 +2778,16 @@
         <v>86</v>
       </c>
       <c r="C35" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D35" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E35" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="F35" t="n">
-        <v>1.0</v>
+        <v>6.0</v>
       </c>
     </row>
     <row r="36">
@@ -2801,13 +2801,13 @@
         <v>104</v>
       </c>
       <c r="D36" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E36" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F36" t="n">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="37">
@@ -2818,16 +2818,16 @@
         <v>88</v>
       </c>
       <c r="C37" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D37" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="E37" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="F37" t="n">
-        <v>1.0</v>
+        <v>43.0</v>
       </c>
     </row>
     <row r="38">
@@ -2844,7 +2844,7 @@
         <v>140</v>
       </c>
       <c r="E38" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F38" t="n">
         <v>1.0</v>
@@ -2864,10 +2864,10 @@
         <v>141</v>
       </c>
       <c r="E39" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F39" t="n">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="40">
@@ -2878,13 +2878,13 @@
         <v>91</v>
       </c>
       <c r="C40" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D40" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E40" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F40" t="n">
         <v>3.0</v>
@@ -2898,13 +2898,13 @@
         <v>92</v>
       </c>
       <c r="C41" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D41" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E41" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F41" t="n">
         <v>1.0</v>
@@ -2921,13 +2921,13 @@
         <v>104</v>
       </c>
       <c r="D42" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E42" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="F42" t="n">
-        <v>3.0</v>
+        <v>10.0</v>
       </c>
     </row>
     <row r="43">
@@ -2941,13 +2941,13 @@
         <v>104</v>
       </c>
       <c r="D43" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="E43" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="F43" t="n">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="44">
@@ -2961,13 +2961,13 @@
         <v>103</v>
       </c>
       <c r="D44" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="E44" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="F44" t="n">
-        <v>6.0</v>
+        <v>13.0</v>
       </c>
     </row>
     <row r="45">
@@ -2981,13 +2981,13 @@
         <v>103</v>
       </c>
       <c r="D45" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="E45" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="F45" t="n">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="46">
@@ -2998,16 +2998,16 @@
         <v>97</v>
       </c>
       <c r="C46" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D46" t="s">
         <v>146</v>
       </c>
       <c r="E46" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F46" t="n">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="47">
@@ -3018,16 +3018,16 @@
         <v>98</v>
       </c>
       <c r="C47" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D47" t="s">
         <v>147</v>
       </c>
       <c r="E47" t="s">
-        <v>189</v>
+        <v>174</v>
       </c>
       <c r="F47" t="n">
-        <v>3.0</v>
+        <v>13.0</v>
       </c>
     </row>
     <row r="48">
@@ -3038,7 +3038,7 @@
         <v>99</v>
       </c>
       <c r="C48" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D48" t="s">
         <v>148</v>
@@ -3047,7 +3047,7 @@
         <v>190</v>
       </c>
       <c r="F48" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="49">
@@ -3058,7 +3058,7 @@
         <v>100</v>
       </c>
       <c r="C49" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D49" t="s">
         <v>149</v>
@@ -3067,7 +3067,7 @@
         <v>191</v>
       </c>
       <c r="F49" t="n">
-        <v>11.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="50">
@@ -3078,7 +3078,7 @@
         <v>101</v>
       </c>
       <c r="C50" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D50" t="s">
         <v>150</v>
@@ -3087,7 +3087,7 @@
         <v>192</v>
       </c>
       <c r="F50" t="n">
-        <v>18.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="51">
@@ -3098,7 +3098,7 @@
         <v>102</v>
       </c>
       <c r="C51" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D51" t="s">
         <v>151</v>
@@ -3140,13 +3140,13 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E2" t="n">
         <v>1.0</v>
@@ -3157,13 +3157,13 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>97</v>
+        <v>59</v>
       </c>
       <c r="C3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D3" t="s">
-        <v>146</v>
+        <v>115</v>
       </c>
       <c r="E3" t="n">
         <v>2.0</v>
@@ -3174,13 +3174,13 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="C4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D4" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="E4" t="n">
         <v>0.0</v>
@@ -3191,13 +3191,13 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D5" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="E5" t="n">
         <v>0.0</v>
@@ -3208,13 +3208,13 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="C6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D6" t="s">
-        <v>121</v>
+        <v>149</v>
       </c>
       <c r="E6" t="n">
         <v>2.0</v>
@@ -3225,13 +3225,13 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>74</v>
+        <v>95</v>
       </c>
       <c r="C7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D7" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="E7" t="n">
         <v>0.0</v>
@@ -3242,13 +3242,13 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D8" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="E8" t="n">
         <v>0.0</v>
@@ -3259,13 +3259,13 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D9" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="E9" t="n">
         <v>2.0</v>
@@ -3276,13 +3276,13 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>99</v>
+        <v>60</v>
       </c>
       <c r="C10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D10" t="s">
-        <v>148</v>
+        <v>116</v>
       </c>
       <c r="E10" t="n">
         <v>0.0</v>
@@ -3293,13 +3293,13 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="C11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D11" t="s">
-        <v>149</v>
+        <v>136</v>
       </c>
       <c r="E11" t="n">
         <v>3.0</v>
@@ -3310,13 +3310,13 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C12" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D12" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="E12" t="n">
         <v>0.0</v>
@@ -3327,13 +3327,13 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="C13" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D13" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="E13" t="n">
         <v>0.0</v>
@@ -3344,13 +3344,13 @@
         <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D14" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="E14" t="n">
         <v>0.0</v>
@@ -3361,13 +3361,13 @@
         <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="C15" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D15" t="s">
-        <v>131</v>
+        <v>146</v>
       </c>
       <c r="E15" t="n">
         <v>0.0</v>
@@ -3378,13 +3378,13 @@
         <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C16" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D16" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E16" t="n">
         <v>0.0</v>
@@ -3395,13 +3395,13 @@
         <v>18</v>
       </c>
       <c r="B17" t="s">
-        <v>53</v>
+        <v>89</v>
       </c>
       <c r="C17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D17" t="s">
-        <v>109</v>
+        <v>140</v>
       </c>
       <c r="E17" t="n">
         <v>0.0</v>
@@ -3412,13 +3412,13 @@
         <v>19</v>
       </c>
       <c r="B18" t="s">
-        <v>54</v>
+        <v>91</v>
       </c>
       <c r="C18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D18" t="s">
-        <v>110</v>
+        <v>142</v>
       </c>
       <c r="E18" t="n">
         <v>0.0</v>
@@ -3429,13 +3429,13 @@
         <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="C19" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D19" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="E19" t="n">
         <v>1.0</v>
@@ -3446,13 +3446,13 @@
         <v>21</v>
       </c>
       <c r="B20" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="C20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D20" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="E20" t="n">
         <v>0.0</v>
@@ -3463,13 +3463,13 @@
         <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="C21" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D21" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="E21" t="n">
         <v>2.0</v>
@@ -3480,13 +3480,13 @@
         <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C22" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D22" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="E22" t="n">
         <v>2.0</v>
@@ -3497,13 +3497,13 @@
         <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>90</v>
+        <v>55</v>
       </c>
       <c r="C23" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D23" t="s">
-        <v>141</v>
+        <v>111</v>
       </c>
       <c r="E23" t="n">
         <v>0.0</v>
@@ -3514,13 +3514,13 @@
         <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="C24" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D24" t="s">
-        <v>141</v>
+        <v>111</v>
       </c>
       <c r="E24" t="n">
         <v>0.0</v>
@@ -3531,13 +3531,13 @@
         <v>26</v>
       </c>
       <c r="B25" t="s">
-        <v>92</v>
+        <v>56</v>
       </c>
       <c r="C25" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D25" t="s">
-        <v>142</v>
+        <v>112</v>
       </c>
       <c r="E25" t="n">
         <v>2.0</v>
@@ -3548,13 +3548,13 @@
         <v>27</v>
       </c>
       <c r="B26" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="C26" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D26" t="s">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="E26" t="n">
         <v>2.0</v>
@@ -3565,13 +3565,13 @@
         <v>28</v>
       </c>
       <c r="B27" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="C27" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D27" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="E27" t="n">
         <v>0.0</v>
@@ -3582,13 +3582,13 @@
         <v>29</v>
       </c>
       <c r="B28" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="C28" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D28" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="E28" t="n">
         <v>0.0</v>
@@ -3599,13 +3599,13 @@
         <v>30</v>
       </c>
       <c r="B29" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="C29" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D29" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="E29" t="n">
         <v>0.0</v>
@@ -3616,13 +3616,13 @@
         <v>31</v>
       </c>
       <c r="B30" t="s">
-        <v>101</v>
+        <v>77</v>
       </c>
       <c r="C30" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D30" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
       <c r="E30" t="n">
         <v>1.0</v>
@@ -3633,13 +3633,13 @@
         <v>32</v>
       </c>
       <c r="B31" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C31" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D31" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E31" t="n">
         <v>1.0</v>
@@ -3650,13 +3650,13 @@
         <v>33</v>
       </c>
       <c r="B32" t="s">
-        <v>88</v>
+        <v>74</v>
       </c>
       <c r="C32" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D32" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="E32" t="n">
         <v>2.0</v>
@@ -3667,13 +3667,13 @@
         <v>34</v>
       </c>
       <c r="B33" t="s">
-        <v>89</v>
+        <v>54</v>
       </c>
       <c r="C33" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D33" t="s">
-        <v>140</v>
+        <v>110</v>
       </c>
       <c r="E33" t="n">
         <v>0.0</v>
@@ -3684,13 +3684,13 @@
         <v>35</v>
       </c>
       <c r="B34" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C34" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D34" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="E34" t="n">
         <v>0.0</v>
@@ -3701,13 +3701,13 @@
         <v>36</v>
       </c>
       <c r="B35" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C35" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D35" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="E35" t="n">
         <v>1.0</v>
@@ -3718,13 +3718,13 @@
         <v>37</v>
       </c>
       <c r="B36" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C36" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D36" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E36" t="n">
         <v>0.0</v>
@@ -3735,13 +3735,13 @@
         <v>38</v>
       </c>
       <c r="B37" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C37" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D37" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E37" t="n">
         <v>0.0</v>
@@ -3752,10 +3752,10 @@
         <v>39</v>
       </c>
       <c r="B38" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C38" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D38" t="s">
         <v>120</v>
@@ -3769,13 +3769,13 @@
         <v>40</v>
       </c>
       <c r="B39" t="s">
-        <v>87</v>
+        <v>53</v>
       </c>
       <c r="C39" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D39" t="s">
-        <v>138</v>
+        <v>109</v>
       </c>
       <c r="E39" t="n">
         <v>0.0</v>
@@ -3786,13 +3786,13 @@
         <v>41</v>
       </c>
       <c r="B40" t="s">
-        <v>61</v>
+        <v>101</v>
       </c>
       <c r="C40" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D40" t="s">
-        <v>116</v>
+        <v>150</v>
       </c>
       <c r="E40" t="n">
         <v>0.0</v>
@@ -3803,13 +3803,13 @@
         <v>42</v>
       </c>
       <c r="B41" t="s">
-        <v>62</v>
+        <v>102</v>
       </c>
       <c r="C41" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D41" t="s">
-        <v>117</v>
+        <v>151</v>
       </c>
       <c r="E41" t="n">
         <v>1.0</v>
@@ -3820,13 +3820,13 @@
         <v>43</v>
       </c>
       <c r="B42" t="s">
-        <v>85</v>
+        <v>57</v>
       </c>
       <c r="C42" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D42" t="s">
-        <v>136</v>
+        <v>113</v>
       </c>
       <c r="E42" t="n">
         <v>2.0</v>
@@ -3837,13 +3837,13 @@
         <v>44</v>
       </c>
       <c r="B43" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="C43" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D43" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="E43" t="n">
         <v>0.0</v>
@@ -3854,13 +3854,13 @@
         <v>45</v>
       </c>
       <c r="B44" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="C44" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D44" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="E44" t="n">
         <v>0.0</v>
@@ -3871,13 +3871,13 @@
         <v>46</v>
       </c>
       <c r="B45" t="s">
-        <v>64</v>
+        <v>92</v>
       </c>
       <c r="C45" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D45" t="s">
-        <v>119</v>
+        <v>143</v>
       </c>
       <c r="E45" t="n">
         <v>0.0</v>
@@ -3888,13 +3888,13 @@
         <v>47</v>
       </c>
       <c r="B46" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="C46" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D46" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="E46" t="n">
         <v>0.0</v>
@@ -3905,13 +3905,13 @@
         <v>48</v>
       </c>
       <c r="B47" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="C47" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D47" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="E47" t="n">
         <v>0.0</v>
@@ -3922,13 +3922,13 @@
         <v>49</v>
       </c>
       <c r="B48" t="s">
-        <v>81</v>
+        <v>98</v>
       </c>
       <c r="C48" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D48" t="s">
-        <v>132</v>
+        <v>147</v>
       </c>
       <c r="E48" t="n">
         <v>2.0</v>
@@ -3939,13 +3939,13 @@
         <v>50</v>
       </c>
       <c r="B49" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C49" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D49" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E49" t="n">
         <v>0.0</v>
@@ -3956,13 +3956,13 @@
         <v>51</v>
       </c>
       <c r="B50" t="s">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="C50" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D50" t="s">
-        <v>143</v>
+        <v>114</v>
       </c>
       <c r="E50" t="n">
         <v>0.0</v>
@@ -3973,13 +3973,13 @@
         <v>52</v>
       </c>
       <c r="B51" t="s">
-        <v>94</v>
+        <v>62</v>
       </c>
       <c r="C51" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D51" t="s">
-        <v>143</v>
+        <v>114</v>
       </c>
       <c r="E51" t="n">
         <v>0.0</v>

</xml_diff>